<commit_message>
Update principal's remark logic for scores 50 and below and update dashboard labels
</commit_message>
<xml_diff>
--- a/Extra_curricular/2025_2026/Second_term/JSS1/extra_jss1_second_term_2025_2026.xlsx
+++ b/Extra_curricular/2025_2026/Second_term/JSS1/extra_jss1_second_term_2025_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Reporter\Extra_curricular\2025_2026\Second_term\JSS1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E70CC3-D483-4759-94EA-84D3FE64CA7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C769CD-1431-4290-8CA5-887B676CBD23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A3584512-35F2-4ADB-935B-FFA0649CF8D6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>Admission_no</t>
   </si>
@@ -105,12 +105,6 @@
     <t>you have proven to be a great student I wish you more success in your endeavours</t>
   </si>
   <si>
-    <t>press club</t>
-  </si>
-  <si>
-    <t>red cross</t>
-  </si>
-  <si>
     <t>nil</t>
   </si>
   <si>
@@ -126,17 +120,53 @@
     <t>days_absent</t>
   </si>
   <si>
-    <t>holiday</t>
+    <t>next_term</t>
+  </si>
+  <si>
+    <t>JESTS Club</t>
+  </si>
+  <si>
+    <t>Boys Scout</t>
+  </si>
+  <si>
+    <t>Qoyum, you have improved greatly from last term, all you need is more of focus, determination and hard and I promise, you will be better than this</t>
+  </si>
+  <si>
+    <t>Lahbeeb, this is an Impressive performance I am very proud of your dilligence and hardwork. All I want as a promise to me is to Improve your Handwriting  coming next-term</t>
+  </si>
+  <si>
+    <t>This is actually an Impressive Performance Sammy!! Keep the candle burning</t>
+  </si>
+  <si>
+    <t>Muhammad I am  very proud of your performance, I want to see more of this and even better than this Next-term</t>
+  </si>
+  <si>
+    <t>Congratulationss!!!, I am very proud of this result, if you want to keep getting more performance like this or even better don’t relent, keep reading always and do assignments regularly</t>
+  </si>
+  <si>
+    <t>4th, May 2026</t>
+  </si>
+  <si>
+    <t>Medical Purpose</t>
+  </si>
+  <si>
+    <t>I believe Tijani has the potential to be an excellent student all he needs is the push from the family so he can Buckle down, he will do better if he is Consistently present and punctual to school and never misses out in important classworks and assignments lastly I want you to improve your Hand-writing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -478,21 +508,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85E5E3D3-9591-4CC7-8F77-1C6A7F21E993}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.36328125" customWidth="1"/>
-    <col min="7" max="7" width="70.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="200.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -500,371 +533,399 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
         <v>29</v>
       </c>
-      <c r="D1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" t="s">
-        <v>4</v>
-      </c>
       <c r="J1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>8</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2">
         <v>100</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>99</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" t="s">
         <v>33</v>
       </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2">
-        <v>5</v>
-      </c>
       <c r="K2">
         <v>4</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O2">
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3">
         <v>100</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>99</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s">
         <v>33</v>
       </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3">
-        <v>5</v>
-      </c>
       <c r="K3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N3">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O3">
+        <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4">
         <v>100</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>99</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
         <v>33</v>
       </c>
-      <c r="G4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4">
-        <v>5</v>
-      </c>
       <c r="K4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N4">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O4">
+        <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5">
         <v>100</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>99</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" t="s">
         <v>33</v>
       </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
       <c r="K5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O5">
+        <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6">
         <v>100</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>99</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" t="s">
         <v>33</v>
       </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
       <c r="K6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6">
         <v>5</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O6">
+        <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>20</v>
       </c>
       <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7">
         <v>100</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>99</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J7" t="s">
         <v>33</v>
       </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
       <c r="K7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N7">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O7">
+        <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>21</v>
       </c>
       <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8">
         <v>100</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>99</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J8" t="s">
         <v>33</v>
       </c>
-      <c r="G8" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I8" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8">
-        <v>5</v>
-      </c>
       <c r="K8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L8">
         <v>5</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N8">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O8">
+        <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
       <c r="B9" t="s">
         <v>24</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9">
         <v>100</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>99</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" t="s">
         <v>33</v>
       </c>
-      <c r="G9" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J9">
-        <v>5</v>
-      </c>
       <c r="K9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N9">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="O9">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
i added the students attendance details days present and absent
</commit_message>
<xml_diff>
--- a/Extra_curricular/2025_2026/Second_term/JSS1/extra_jss1_second_term_2025_2026.xlsx
+++ b/Extra_curricular/2025_2026/Second_term/JSS1/extra_jss1_second_term_2025_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Reporter\Extra_curricular\2025_2026\Second_term\JSS1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C769CD-1431-4290-8CA5-887B676CBD23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04349AEC-FFE8-4BE0-92C5-6DBFF6A29A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A3584512-35F2-4ADB-935B-FFA0649CF8D6}"/>
   </bookViews>
@@ -583,10 +583,13 @@
         <v>39</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E2">
-        <v>99</v>
+        <v>65</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
       </c>
       <c r="G2" t="s">
         <v>26</v>
@@ -627,10 +630,13 @@
         <v>39</v>
       </c>
       <c r="D3">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E3">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
       </c>
       <c r="G3" t="s">
         <v>26</v>
@@ -671,10 +677,13 @@
         <v>39</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E4">
-        <v>99</v>
+        <v>66</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
       </c>
       <c r="G4" t="s">
         <v>26</v>
@@ -715,10 +724,7 @@
         <v>39</v>
       </c>
       <c r="D5">
-        <v>100</v>
-      </c>
-      <c r="E5">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="G5" t="s">
         <v>26</v>
@@ -759,10 +765,13 @@
         <v>39</v>
       </c>
       <c r="D6">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E6">
-        <v>99</v>
+        <v>62</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
       </c>
       <c r="G6" t="s">
         <v>26</v>
@@ -803,10 +812,13 @@
         <v>39</v>
       </c>
       <c r="D7">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E7">
-        <v>99</v>
+        <v>56</v>
+      </c>
+      <c r="F7">
+        <v>11</v>
       </c>
       <c r="G7" t="s">
         <v>40</v>
@@ -847,10 +859,13 @@
         <v>39</v>
       </c>
       <c r="D8">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E8">
-        <v>99</v>
+        <v>52</v>
+      </c>
+      <c r="F8">
+        <v>15</v>
       </c>
       <c r="G8" t="s">
         <v>26</v>
@@ -891,10 +906,13 @@
         <v>39</v>
       </c>
       <c r="D9">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="E9">
-        <v>99</v>
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
       </c>
       <c r="G9" t="s">
         <v>26</v>

</xml_diff>